<commit_message>
Align public release with current manuscript and SI
</commit_message>
<xml_diff>
--- a/Source_Data.xlsx
+++ b/Source_Data.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2cb7fdd6b3b044fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_2" sheetId="2" r:id="Rb82f8005f76a453f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_3" sheetId="3" r:id="R4551f058a0854c2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_4" sheetId="4" r:id="R479df79f67214771"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_5" sheetId="5" r:id="Rf3f21958631d4a71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_6" sheetId="6" r:id="R01b1770d27454fee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp_Fig_S1" sheetId="7" r:id="Ra70ec4d94136410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp_Fig_S2" sheetId="8" r:id="Ra26590d5584a4387"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numeric_Tests" sheetId="9" r:id="R1099dbd9af8a4e54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Data_Summary" sheetId="10" r:id="Rc80d43d1c217412d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort_Metadata" sheetId="11" r:id="R6026e5bdaf614d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Map" sheetId="12" r:id="R287e231829914625"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Dictionary" sheetId="13" r:id="Re6eda02dfcf24e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp_Table_S1" sheetId="14" r:id="R5ee87902028c42cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R881ffe375d5644da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_2" sheetId="2" r:id="R4e9b5b4ab4c043e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_3" sheetId="3" r:id="R4f5868f09e554bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_4" sheetId="4" r:id="R1f3a7322ae454cfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_5" sheetId="5" r:id="R0ced5ab308814992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fig_6" sheetId="6" r:id="Re6d4e9df6ae545ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp_Fig_S1" sheetId="7" r:id="R6e4347879c464b27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp_Fig_S2" sheetId="8" r:id="Rc3037ebff36a4672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numeric_Tests" sheetId="9" r:id="R4387f64a61d540a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_Data_Summary" sheetId="10" r:id="R45bb2903874946e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort_Metadata" sheetId="11" r:id="Ra01c25c345004f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Map" sheetId="12" r:id="R2808decdb8874a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Dictionary" sheetId="13" r:id="R893fc537cf274641"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supp_Table_S1" sheetId="14" r:id="Refb747b4557d49a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,8 +26,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.0000"/>
+    <x:numFmt numFmtId="201" formatCode="0.000000"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -50,7 +51,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -60,6 +61,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -169,7 +180,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -247,6 +258,33 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -716,12 +754,12 @@
         <x:v>description</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="36" hidden="0" customHeight="1">
+    <x:row r="2" ht="48" hidden="0" customHeight="1">
       <x:c r="A2" s="1" t="str">
         <x:v>Scope</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>Aggregate numerical source data underlying revised Figs. 2-6, Supplementary Figs. S1-S2, Supplementary Table S1, and synthetic transition-boundary tests.</x:v>
+        <x:v>Aggregate numerical source data underlying revised Figs. 2-6, current Supplementary Table S1, a privacy-safe aggregate companion to Supplementary Fig. S1, repository-only boundary analyses, and synthetic transition-boundary tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="24" hidden="0" customHeight="1">
@@ -748,12 +786,12 @@
         <x:v>No real or coded participant, seizure, channel, electrode, or contact identifiers are included.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="24" hidden="0" customHeight="1">
+    <x:row r="6" ht="36" hidden="0" customHeight="1">
       <x:c r="A6" s="1" t="str">
         <x:v>Explicit exclusions</x:v>
       </x:c>
       <x:c r="B6" s="5" t="str">
-        <x:v>No raw SEEG, clinical labels, coordinates, dates, institutional identifiers, linkage keys, local paths, or participant-derived rows.</x:v>
+        <x:v>No raw SEEG, participant-level rows, clinical labels, coordinates, dates, institutional identifiers, linkage keys, local paths, manuscript files, or personal contact metadata.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -780,18 +818,18 @@
         <x:v>Restricted human-participant data remain governed by the originating ethics, consent, institutional, and clinical data-use conditions.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="24" hidden="0" customHeight="1">
+    <x:row r="10" ht="36" hidden="0" customHeight="1">
       <x:c r="A10" s="1" t="str">
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>Public aggregate release synchronized on 2026-08-21 with the current JBHI submission manuscript.</x:v>
+        <x:v>Public aggregate release synchronized on 2026-08-22 with the current JBHI manuscript and SI; patient-level Supplementary Table S2 and Supplementary Fig. S1 points are withheld.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2af5bc2367544ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce569af32988410f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -852,7 +890,7 @@
       <x:c r="E2" s="5" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="str">
+      <x:c r="F2" s="5" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G2" s="5" t="str">
@@ -878,7 +916,7 @@
       <x:c r="E3" s="5" t="str">
         <x:v>Methods description only</x:v>
       </x:c>
-      <x:c r="F3" s="1" t="str">
+      <x:c r="F3" s="5" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G3" s="5" t="str">
@@ -904,7 +942,7 @@
       <x:c r="E4" s="5" t="str">
         <x:v>Aggregate estimates and intervals</x:v>
       </x:c>
-      <x:c r="F4" s="1" t="str">
+      <x:c r="F4" s="5" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="G4" s="5" t="str">
@@ -914,7 +952,7 @@
         <x:v>Small-cohort linkage and attribute-disclosure risk.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="5" t="str">
         <x:v>Aggregate analysis outputs</x:v>
       </x:c>
@@ -928,9 +966,9 @@
         <x:v>cohort aggregate</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>Fig_2 through Supp_Fig_S2</x:v>
-      </x:c>
-      <x:c r="F5" s="1" t="str">
+        <x:v>Figs. 2-6, aggregate Supplementary Table S1, aggregate companion to Supplementary Fig. S1, and repository-only boundary checks</x:v>
+      </x:c>
+      <x:c r="F5" s="5" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
@@ -956,7 +994,7 @@
       <x:c r="E6" s="5" t="str">
         <x:v>examples, tests, Numeric_Tests</x:v>
       </x:c>
-      <x:c r="F6" s="1" t="str">
+      <x:c r="F6" s="5" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G6" s="5" t="str">
@@ -969,7 +1007,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba7a21a94c8d4729"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb53c93b41b5649b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1158,7 +1196,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc78c19b0bf343a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9263db1f8a2b4cf6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1168,64 +1206,64 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="62" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="70" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="8" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="23" t="str">
+      <x:c r="A1" s="46" t="str">
         <x:v>worksheet</x:v>
       </x:c>
-      <x:c r="B1" s="24" t="str">
+      <x:c r="B1" s="47" t="str">
         <x:v>figure_or_table</x:v>
       </x:c>
-      <x:c r="C1" s="24" t="str">
+      <x:c r="C1" s="47" t="str">
         <x:v>panel</x:v>
       </x:c>
-      <x:c r="D1" s="24" t="str">
+      <x:c r="D1" s="47" t="str">
         <x:v>contents</x:v>
       </x:c>
-      <x:c r="E1" s="24" t="str">
+      <x:c r="E1" s="47" t="str">
         <x:v>analysis_unit</x:v>
       </x:c>
-      <x:c r="F1" s="24" t="str">
+      <x:c r="F1" s="47" t="str">
         <x:v>data_range</x:v>
       </x:c>
-      <x:c r="G1" s="24" t="str">
+      <x:c r="G1" s="47" t="str">
         <x:v>rows</x:v>
       </x:c>
-      <x:c r="H1" s="24" t="str">
+      <x:c r="H1" s="47" t="str">
         <x:v>privacy_level</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="24" hidden="0" customHeight="1">
-      <x:c r="A2" s="26" t="str">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="49" t="str">
         <x:v>Fig_2</x:v>
       </x:c>
-      <x:c r="B2" s="27" t="str">
+      <x:c r="B2" s="59" t="str">
         <x:v>Fig. 2</x:v>
       </x:c>
-      <x:c r="C2" s="27" t="str">
+      <x:c r="C2" s="59" t="str">
         <x:v>e-h</x:v>
       </x:c>
-      <x:c r="D2" s="40" t="str">
+      <x:c r="D2" s="59" t="str">
         <x:v>Regional node activity, benchmark AP, label-permutation lift, AUROC, and enrichment.</x:v>
       </x:c>
-      <x:c r="E2" s="27" t="str">
-        <x:v>cohort aggregate</x:v>
-      </x:c>
-      <x:c r="F2" s="27" t="str">
+      <x:c r="E2" s="59" t="str">
+        <x:v>cohort aggregate</x:v>
+      </x:c>
+      <x:c r="F2" s="50" t="str">
         <x:v>A1:Q18</x:v>
       </x:c>
-      <x:c r="G2" s="27" t="n">
+      <x:c r="G2" s="50" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="H2" s="28" t="str">
+      <x:c r="H2" s="51" t="str">
         <x:v>aggregate only</x:v>
       </x:c>
     </x:row>
@@ -1233,16 +1271,16 @@
       <x:c r="A3" s="14" t="str">
         <x:v>Fig_3</x:v>
       </x:c>
-      <x:c r="B3" s="15" t="str">
+      <x:c r="B3" s="41" t="str">
         <x:v>Fig. 3</x:v>
       </x:c>
-      <x:c r="C3" s="15" t="str">
+      <x:c r="C3" s="41" t="str">
         <x:v>aggregate</x:v>
       </x:c>
       <x:c r="D3" s="41" t="str">
         <x:v>Ictal-minus-pre transition concentration by region.</x:v>
       </x:c>
-      <x:c r="E3" s="15" t="str">
+      <x:c r="E3" s="41" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
       <x:c r="F3" s="15" t="str">
@@ -1256,28 +1294,28 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="26" t="str">
+      <x:c r="A4" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B4" s="27" t="str">
+      <x:c r="B4" s="59" t="str">
         <x:v>Fig. 4</x:v>
       </x:c>
-      <x:c r="C4" s="27" t="str">
+      <x:c r="C4" s="59" t="str">
         <x:v>b–c</x:v>
       </x:c>
-      <x:c r="D4" s="40" t="str">
+      <x:c r="D4" s="59" t="str">
         <x:v>Dynamic module stability and entropy changes.</x:v>
       </x:c>
-      <x:c r="E4" s="27" t="str">
+      <x:c r="E4" s="59" t="str">
         <x:v>paired cohort aggregate</x:v>
       </x:c>
-      <x:c r="F4" s="27" t="str">
+      <x:c r="F4" s="50" t="str">
         <x:v>A1:P9</x:v>
       </x:c>
-      <x:c r="G4" s="27" t="n">
+      <x:c r="G4" s="50" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="H4" s="28" t="str">
+      <x:c r="H4" s="51" t="str">
         <x:v>aggregate only</x:v>
       </x:c>
     </x:row>
@@ -1285,16 +1323,16 @@
       <x:c r="A5" s="14" t="str">
         <x:v>Fig_5</x:v>
       </x:c>
-      <x:c r="B5" s="15" t="str">
+      <x:c r="B5" s="41" t="str">
         <x:v>Fig. 5</x:v>
       </x:c>
-      <x:c r="C5" s="15" t="str">
+      <x:c r="C5" s="41" t="str">
         <x:v>b–d</x:v>
       </x:c>
       <x:c r="D5" s="41" t="str">
         <x:v>Attribute/topology contrasts and projection efficiency.</x:v>
       </x:c>
-      <x:c r="E5" s="15" t="str">
+      <x:c r="E5" s="41" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
       <x:c r="F5" s="15" t="str">
@@ -1308,45 +1346,45 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="26" t="str">
+      <x:c r="A6" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B6" s="27" t="str">
+      <x:c r="B6" s="59" t="str">
         <x:v>Fig. 6</x:v>
       </x:c>
-      <x:c r="C6" s="27" t="str">
+      <x:c r="C6" s="59" t="str">
         <x:v>a–c</x:v>
       </x:c>
-      <x:c r="D6" s="40" t="str">
+      <x:c r="D6" s="59" t="str">
         <x:v>Sensitivity configurations and jump-strategy stability.</x:v>
       </x:c>
-      <x:c r="E6" s="27" t="str">
-        <x:v>cohort aggregate</x:v>
-      </x:c>
-      <x:c r="F6" s="27" t="str">
+      <x:c r="E6" s="59" t="str">
+        <x:v>cohort aggregate</x:v>
+      </x:c>
+      <x:c r="F6" s="50" t="str">
         <x:v>A1:R32</x:v>
       </x:c>
-      <x:c r="G6" s="27" t="n">
+      <x:c r="G6" s="50" t="n">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="H6" s="28" t="str">
+      <x:c r="H6" s="51" t="str">
         <x:v>aggregate only</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+    <x:row r="7" ht="24" hidden="0" customHeight="1">
       <x:c r="A7" s="14" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B7" s="15" t="str">
-        <x:v>Supplementary Fig. S1</x:v>
-      </x:c>
-      <x:c r="C7" s="15" t="str">
-        <x:v>aggregate</x:v>
+      <x:c r="B7" s="41" t="str">
+        <x:v>Supplementary Fig. S1 aggregate companion</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="str">
+        <x:v>configuration summary</x:v>
       </x:c>
       <x:c r="D7" s="41" t="str">
-        <x:v>Configuration-level sensitivity summary.</x:v>
-      </x:c>
-      <x:c r="E7" s="15" t="str">
+        <x:v>Privacy-safe aggregate companion; patient-level points in the submitted SI figure are withheld.</x:v>
+      </x:c>
+      <x:c r="E7" s="41" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
       <x:c r="F7" s="15" t="str">
@@ -1359,29 +1397,29 @@
         <x:v>aggregate only</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="26" t="str">
+    <x:row r="8" ht="24" hidden="0" customHeight="1">
+      <x:c r="A8" s="49" t="str">
         <x:v>Supp_Table_S1</x:v>
       </x:c>
-      <x:c r="B8" s="27" t="str">
+      <x:c r="B8" s="59" t="str">
         <x:v>Supplementary Table S1</x:v>
       </x:c>
-      <x:c r="C8" s="27" t="str">
-        <x:v>complete</x:v>
-      </x:c>
-      <x:c r="D8" s="40" t="str">
-        <x:v>Paired AP differences against benchmark controls.</x:v>
-      </x:c>
-      <x:c r="E8" s="27" t="str">
-        <x:v>paired cohort aggregate</x:v>
-      </x:c>
-      <x:c r="F8" s="27" t="str">
-        <x:v>A1:M5</x:v>
-      </x:c>
-      <x:c r="G8" s="27" t="n">
+      <x:c r="C8" s="59" t="str">
+        <x:v>complete aggregate table</x:v>
+      </x:c>
+      <x:c r="D8" s="59" t="str">
+        <x:v>HyNaPT reference plus three aggregate benchmark comparisons; patient-level Table S2 is withheld.</x:v>
+      </x:c>
+      <x:c r="E8" s="59" t="str">
+        <x:v>cohort/paired cohort aggregate</x:v>
+      </x:c>
+      <x:c r="F8" s="50" t="str">
+        <x:v>A1:J5</x:v>
+      </x:c>
+      <x:c r="G8" s="50" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="H8" s="28" t="str">
+      <x:c r="H8" s="51" t="str">
         <x:v>aggregate only</x:v>
       </x:c>
     </x:row>
@@ -1389,16 +1427,16 @@
       <x:c r="A9" s="14" t="str">
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
-      <x:c r="B9" s="15" t="str">
-        <x:v>Supplementary Fig. S2</x:v>
-      </x:c>
-      <x:c r="C9" s="15" t="str">
-        <x:v>a–c</x:v>
+      <x:c r="B9" s="41" t="str">
+        <x:v>Repository-only boundary analyses</x:v>
+      </x:c>
+      <x:c r="C9" s="41" t="str">
+        <x:v>historical worksheet name</x:v>
       </x:c>
       <x:c r="D9" s="41" t="str">
-        <x:v>Aggregate null and boundary analyses.</x:v>
-      </x:c>
-      <x:c r="E9" s="15" t="str">
+        <x:v>Additional aggregate null and boundary analyses; not a figure in the current SI.</x:v>
+      </x:c>
+      <x:c r="E9" s="41" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
       <x:c r="F9" s="15" t="str">
@@ -1412,28 +1450,28 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="26" t="str">
+      <x:c r="A10" s="49" t="str">
         <x:v>Numeric_Tests</x:v>
       </x:c>
-      <x:c r="B10" s="27" t="str">
+      <x:c r="B10" s="59" t="str">
         <x:v>Transition tests</x:v>
       </x:c>
-      <x:c r="C10" s="27" t="str">
+      <x:c r="C10" s="59" t="str">
         <x:v>complete</x:v>
       </x:c>
-      <x:c r="D10" s="40" t="str">
+      <x:c r="D10" s="59" t="str">
         <x:v>Synthetic normalization, isolation, asymmetry, fusion, and path checks.</x:v>
       </x:c>
-      <x:c r="E10" s="27" t="str">
+      <x:c r="E10" s="59" t="str">
         <x:v>synthetic test</x:v>
       </x:c>
-      <x:c r="F10" s="27" t="str">
+      <x:c r="F10" s="50" t="str">
         <x:v>A1:E10</x:v>
       </x:c>
-      <x:c r="G10" s="27" t="n">
+      <x:c r="G10" s="50" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="H10" s="28" t="str">
+      <x:c r="H10" s="51" t="str">
         <x:v>synthetic</x:v>
       </x:c>
     </x:row>
@@ -1441,16 +1479,16 @@
       <x:c r="A11" s="14" t="str">
         <x:v>Raw_Data_Summary</x:v>
       </x:c>
-      <x:c r="B11" s="15" t="str">
+      <x:c r="B11" s="41" t="str">
         <x:v>Data inventory</x:v>
       </x:c>
-      <x:c r="C11" s="15" t="str">
+      <x:c r="C11" s="41" t="str">
         <x:v>complete</x:v>
       </x:c>
       <x:c r="D11" s="41" t="str">
         <x:v>Public/restricted data-class summary without raw records.</x:v>
       </x:c>
-      <x:c r="E11" s="15" t="str">
+      <x:c r="E11" s="41" t="str">
         <x:v>data class</x:v>
       </x:c>
       <x:c r="F11" s="15" t="str">
@@ -1464,35 +1502,35 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="29" t="str">
+      <x:c r="A12" s="56" t="str">
         <x:v>Cohort_Metadata</x:v>
       </x:c>
-      <x:c r="B12" s="30" t="str">
+      <x:c r="B12" s="60" t="str">
         <x:v>Design metadata</x:v>
       </x:c>
-      <x:c r="C12" s="30" t="str">
+      <x:c r="C12" s="60" t="str">
         <x:v>complete</x:v>
       </x:c>
-      <x:c r="D12" s="42" t="str">
+      <x:c r="D12" s="60" t="str">
         <x:v>Aggregate cohort and analysis-design metadata.</x:v>
       </x:c>
-      <x:c r="E12" s="30" t="str">
+      <x:c r="E12" s="60" t="str">
         <x:v>aggregate/design</x:v>
       </x:c>
-      <x:c r="F12" s="30" t="str">
+      <x:c r="F12" s="57" t="str">
         <x:v>A1:E10</x:v>
       </x:c>
-      <x:c r="G12" s="30" t="n">
+      <x:c r="G12" s="57" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="H12" s="31" t="str">
+      <x:c r="H12" s="58" t="str">
         <x:v>aggregate only</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2cb9035b9a14305"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77248a6f19264980"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1502,176 +1540,176 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="72" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="76" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="23" t="str">
+      <x:c r="A1" s="46" t="str">
         <x:v>worksheet</x:v>
       </x:c>
-      <x:c r="B1" s="24" t="str">
+      <x:c r="B1" s="47" t="str">
         <x:v>variable</x:v>
       </x:c>
-      <x:c r="C1" s="24" t="str">
+      <x:c r="C1" s="47" t="str">
         <x:v>definition</x:v>
       </x:c>
-      <x:c r="D1" s="24" t="str">
+      <x:c r="D1" s="47" t="str">
         <x:v>release_level</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="26" t="str">
-        <x:v>Fig_2</x:v>
-      </x:c>
-      <x:c r="B2" s="27" t="str">
-        <x:v>panel</x:v>
-      </x:c>
-      <x:c r="C2" s="40" t="str">
-        <x:v>Panel identifier in the revised figure.</x:v>
-      </x:c>
-      <x:c r="D2" s="28" t="str">
+      <x:c r="A2" s="49" t="str">
+        <x:v>Supp_Table_S1</x:v>
+      </x:c>
+      <x:c r="B2" s="50" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="C2" s="59" t="str">
+        <x:v>Model row in the current Supplementary Table S1.</x:v>
+      </x:c>
+      <x:c r="D2" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Fig_2</x:v>
+        <x:v>Supp_Table_S1</x:v>
       </x:c>
       <x:c r="B3" s="15" t="str">
-        <x:v>outcome</x:v>
+        <x:v>mean_ap</x:v>
       </x:c>
       <x:c r="C3" s="41" t="str">
-        <x:v>Reported endpoint.</x:v>
+        <x:v>Released cohort mean average precision.</x:v>
       </x:c>
       <x:c r="D3" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="26" t="str">
-        <x:v>Fig_2</x:v>
-      </x:c>
-      <x:c r="B4" s="27" t="str">
-        <x:v>stage</x:v>
-      </x:c>
-      <x:c r="C4" s="40" t="str">
-        <x:v>Seizure-stage aggregate represented by the row.</x:v>
-      </x:c>
-      <x:c r="D4" s="28" t="str">
+      <x:c r="A4" s="49" t="str">
+        <x:v>Supp_Table_S1</x:v>
+      </x:c>
+      <x:c r="B4" s="50" t="str">
+        <x:v>delta_ap</x:v>
+      </x:c>
+      <x:c r="C4" s="59" t="str">
+        <x:v>Mean paired AP difference, HyNaPT minus comparator; blank for the reference row.</x:v>
+      </x:c>
+      <x:c r="D4" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="14" t="str">
-        <x:v>Fig_2</x:v>
+        <x:v>Supp_Table_S1</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>region</x:v>
+        <x:v>ci_low</x:v>
       </x:c>
       <x:c r="C5" s="41" t="str">
-        <x:v>Clinical region category summarized only at cohort level.</x:v>
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="26" t="str">
-        <x:v>Fig_2</x:v>
-      </x:c>
-      <x:c r="B6" s="27" t="str">
-        <x:v>series</x:v>
-      </x:c>
-      <x:c r="C6" s="40" t="str">
-        <x:v>Method, configuration, or stage represented by the row.</x:v>
-      </x:c>
-      <x:c r="D6" s="28" t="str">
+      <x:c r="A6" s="49" t="str">
+        <x:v>Supp_Table_S1</x:v>
+      </x:c>
+      <x:c r="B6" s="50" t="str">
+        <x:v>ci_high</x:v>
+      </x:c>
+      <x:c r="C6" s="59" t="str">
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D6" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="14" t="str">
-        <x:v>Fig_2</x:v>
+        <x:v>Supp_Table_S1</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:v>comparator</x:v>
+        <x:v>exact_p</x:v>
       </x:c>
       <x:c r="C7" s="41" t="str">
-        <x:v>Comparator or null model for the reported contrast.</x:v>
+        <x:v>Two-sided exact sign-flip P value for the paired contrast.</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="26" t="str">
-        <x:v>Fig_2</x:v>
-      </x:c>
-      <x:c r="B8" s="27" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="C8" s="40" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
-      </x:c>
-      <x:c r="D8" s="28" t="str">
+      <x:c r="A8" s="49" t="str">
+        <x:v>Supp_Table_S1</x:v>
+      </x:c>
+      <x:c r="B8" s="50" t="str">
+        <x:v>bh_p</x:v>
+      </x:c>
+      <x:c r="C8" s="59" t="str">
+        <x:v>Benjamini-Hochberg adjusted P value across the three comparator rows.</x:v>
+      </x:c>
+      <x:c r="D8" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="14" t="str">
-        <x:v>Fig_2</x:v>
+        <x:v>Supp_Table_S1</x:v>
       </x:c>
       <x:c r="B9" s="15" t="str">
-        <x:v>sd</x:v>
+        <x:v>n</x:v>
       </x:c>
       <x:c r="C9" s="41" t="str">
-        <x:v>Between-participant standard deviation.</x:v>
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="26" t="str">
-        <x:v>Fig_2</x:v>
-      </x:c>
-      <x:c r="B10" s="27" t="str">
-        <x:v>ci_low</x:v>
-      </x:c>
-      <x:c r="C10" s="40" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D10" s="28" t="str">
+      <x:c r="A10" s="49" t="str">
+        <x:v>Supp_Table_S1</x:v>
+      </x:c>
+      <x:c r="B10" s="50" t="str">
+        <x:v>analysis_unit</x:v>
+      </x:c>
+      <x:c r="C10" s="59" t="str">
+        <x:v>Unit represented by the released row.</x:v>
+      </x:c>
+      <x:c r="D10" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="14" t="str">
+        <x:v>Supp_Table_S1</x:v>
+      </x:c>
+      <x:c r="B11" s="15" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C11" s="41" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D11" s="16" t="str">
+        <x:v>cohort aggregate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="49" t="str">
         <x:v>Fig_2</x:v>
       </x:c>
-      <x:c r="B11" s="15" t="str">
-        <x:v>ci_high</x:v>
-      </x:c>
-      <x:c r="C11" s="41" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D11" s="16" t="str">
-        <x:v>cohort aggregate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="26" t="str">
-        <x:v>Fig_2</x:v>
-      </x:c>
-      <x:c r="B12" s="27" t="str">
-        <x:v>reference</x:v>
-      </x:c>
-      <x:c r="C12" s="40" t="str">
-        <x:v>Null or reference value shown in the panel.</x:v>
-      </x:c>
-      <x:c r="D12" s="28" t="str">
+      <x:c r="B12" s="50" t="str">
+        <x:v>panel</x:v>
+      </x:c>
+      <x:c r="C12" s="59" t="str">
+        <x:v>Panel identifier in the revised figure.</x:v>
+      </x:c>
+      <x:c r="D12" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -1680,26 +1718,26 @@
         <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B13" s="15" t="str">
-        <x:v>p_value</x:v>
+        <x:v>outcome</x:v>
       </x:c>
       <x:c r="C13" s="41" t="str">
-        <x:v>Two-sided exact or joint-permutation P value where applicable.</x:v>
+        <x:v>Reported endpoint.</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="26" t="str">
+      <x:c r="A14" s="49" t="str">
         <x:v>Fig_2</x:v>
       </x:c>
-      <x:c r="B14" s="27" t="str">
-        <x:v>adjusted_p</x:v>
-      </x:c>
-      <x:c r="C14" s="40" t="str">
-        <x:v>Benjamini-Hochberg adjusted P value where applicable.</x:v>
-      </x:c>
-      <x:c r="D14" s="28" t="str">
+      <x:c r="B14" s="50" t="str">
+        <x:v>stage</x:v>
+      </x:c>
+      <x:c r="C14" s="59" t="str">
+        <x:v>Seizure-stage aggregate represented by the row.</x:v>
+      </x:c>
+      <x:c r="D14" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -1708,26 +1746,26 @@
         <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B15" s="15" t="str">
-        <x:v>n</x:v>
+        <x:v>region</x:v>
       </x:c>
       <x:c r="C15" s="41" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+        <x:v>Clinical region category summarized only at cohort level.</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="26" t="str">
+      <x:c r="A16" s="49" t="str">
         <x:v>Fig_2</x:v>
       </x:c>
-      <x:c r="B16" s="27" t="str">
-        <x:v>positive_count</x:v>
-      </x:c>
-      <x:c r="C16" s="40" t="str">
-        <x:v>Number of participants with positive raw lift.</x:v>
-      </x:c>
-      <x:c r="D16" s="28" t="str">
+      <x:c r="B16" s="50" t="str">
+        <x:v>series</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>Method, configuration, or stage represented by the row.</x:v>
+      </x:c>
+      <x:c r="D16" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -1736,222 +1774,222 @@
         <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B17" s="15" t="str">
-        <x:v>analysis_unit</x:v>
+        <x:v>comparator</x:v>
       </x:c>
       <x:c r="C17" s="41" t="str">
-        <x:v>Unit represented by the released row.</x:v>
+        <x:v>Comparator or null model for the reported contrast.</x:v>
       </x:c>
       <x:c r="D17" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="26" t="str">
+      <x:c r="A18" s="49" t="str">
         <x:v>Fig_2</x:v>
       </x:c>
-      <x:c r="B18" s="27" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="C18" s="40" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
-      </x:c>
-      <x:c r="D18" s="28" t="str">
+      <x:c r="B18" s="50" t="str">
+        <x:v>estimate</x:v>
+      </x:c>
+      <x:c r="C18" s="59" t="str">
+        <x:v>Released cohort-level point estimate.</x:v>
+      </x:c>
+      <x:c r="D18" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B19" s="15" t="str">
-        <x:v>outcome</x:v>
+        <x:v>sd</x:v>
       </x:c>
       <x:c r="C19" s="41" t="str">
-        <x:v>Reported endpoint.</x:v>
+        <x:v>Between-participant standard deviation.</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="26" t="str">
-        <x:v>Supp_Table_S1</x:v>
-      </x:c>
-      <x:c r="B20" s="27" t="str">
-        <x:v>series</x:v>
-      </x:c>
-      <x:c r="C20" s="40" t="str">
-        <x:v>Primary model in the paired contrast.</x:v>
-      </x:c>
-      <x:c r="D20" s="28" t="str">
+      <x:c r="A20" s="49" t="str">
+        <x:v>Fig_2</x:v>
+      </x:c>
+      <x:c r="B20" s="50" t="str">
+        <x:v>ci_low</x:v>
+      </x:c>
+      <x:c r="C20" s="59" t="str">
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D20" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B21" s="15" t="str">
-        <x:v>comparator</x:v>
+        <x:v>ci_high</x:v>
       </x:c>
       <x:c r="C21" s="41" t="str">
-        <x:v>Benchmark comparator.</x:v>
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D21" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="26" t="str">
-        <x:v>Supp_Table_S1</x:v>
-      </x:c>
-      <x:c r="B22" s="27" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="C22" s="40" t="str">
-        <x:v>Mean paired participant-level AP difference.</x:v>
-      </x:c>
-      <x:c r="D22" s="28" t="str">
+      <x:c r="A22" s="49" t="str">
+        <x:v>Fig_2</x:v>
+      </x:c>
+      <x:c r="B22" s="50" t="str">
+        <x:v>reference</x:v>
+      </x:c>
+      <x:c r="C22" s="59" t="str">
+        <x:v>Null or reference value shown in the panel.</x:v>
+      </x:c>
+      <x:c r="D22" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B23" s="15" t="str">
-        <x:v>ci_low</x:v>
+        <x:v>p_value</x:v>
       </x:c>
       <x:c r="C23" s="41" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Two-sided exact or joint-permutation P value where applicable.</x:v>
       </x:c>
       <x:c r="D23" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="26" t="str">
-        <x:v>Supp_Table_S1</x:v>
-      </x:c>
-      <x:c r="B24" s="27" t="str">
-        <x:v>ci_high</x:v>
-      </x:c>
-      <x:c r="C24" s="40" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D24" s="28" t="str">
+      <x:c r="A24" s="49" t="str">
+        <x:v>Fig_2</x:v>
+      </x:c>
+      <x:c r="B24" s="50" t="str">
+        <x:v>adjusted_p</x:v>
+      </x:c>
+      <x:c r="C24" s="59" t="str">
+        <x:v>Benjamini-Hochberg adjusted P value where applicable.</x:v>
+      </x:c>
+      <x:c r="D24" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B25" s="15" t="str">
-        <x:v>reference</x:v>
+        <x:v>n</x:v>
       </x:c>
       <x:c r="C25" s="41" t="str">
-        <x:v>Null or reference value shown in the panel.</x:v>
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
       </x:c>
       <x:c r="D25" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="26" t="str">
-        <x:v>Supp_Table_S1</x:v>
-      </x:c>
-      <x:c r="B26" s="27" t="str">
-        <x:v>p_value</x:v>
-      </x:c>
-      <x:c r="C26" s="40" t="str">
-        <x:v>Two-sided exact sign-flip P value.</x:v>
-      </x:c>
-      <x:c r="D26" s="28" t="str">
+      <x:c r="A26" s="49" t="str">
+        <x:v>Fig_2</x:v>
+      </x:c>
+      <x:c r="B26" s="50" t="str">
+        <x:v>positive_count</x:v>
+      </x:c>
+      <x:c r="C26" s="59" t="str">
+        <x:v>Number of participants with positive raw lift.</x:v>
+      </x:c>
+      <x:c r="D26" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_2</x:v>
       </x:c>
       <x:c r="B27" s="15" t="str">
-        <x:v>adjusted_p</x:v>
+        <x:v>analysis_unit</x:v>
       </x:c>
       <x:c r="C27" s="41" t="str">
-        <x:v>Benjamini-Hochberg adjusted P value where applicable.</x:v>
+        <x:v>Unit represented by the released row.</x:v>
       </x:c>
       <x:c r="D27" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="26" t="str">
-        <x:v>Supp_Table_S1</x:v>
-      </x:c>
-      <x:c r="B28" s="27" t="str">
-        <x:v>n</x:v>
-      </x:c>
-      <x:c r="C28" s="40" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
-      </x:c>
-      <x:c r="D28" s="28" t="str">
+      <x:c r="A28" s="49" t="str">
+        <x:v>Fig_2</x:v>
+      </x:c>
+      <x:c r="B28" s="50" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C28" s="59" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D28" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_3</x:v>
       </x:c>
       <x:c r="B29" s="15" t="str">
-        <x:v>analysis_unit</x:v>
+        <x:v>panel</x:v>
       </x:c>
       <x:c r="C29" s="41" t="str">
-        <x:v>Unit represented by the released row.</x:v>
+        <x:v>Panel identifier in the revised figure.</x:v>
       </x:c>
       <x:c r="D29" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="26" t="str">
-        <x:v>Supp_Table_S1</x:v>
-      </x:c>
-      <x:c r="B30" s="27" t="str">
-        <x:v>test</x:v>
-      </x:c>
-      <x:c r="C30" s="40" t="str">
-        <x:v>Statistical test used for the released comparison.</x:v>
-      </x:c>
-      <x:c r="D30" s="28" t="str">
+      <x:c r="A30" s="49" t="str">
+        <x:v>Fig_3</x:v>
+      </x:c>
+      <x:c r="B30" s="50" t="str">
+        <x:v>metric</x:v>
+      </x:c>
+      <x:c r="C30" s="59" t="str">
+        <x:v>Quantity summarized by the row.</x:v>
+      </x:c>
+      <x:c r="D30" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="14" t="str">
-        <x:v>Supp_Table_S1</x:v>
+        <x:v>Fig_3</x:v>
       </x:c>
       <x:c r="B31" s="15" t="str">
-        <x:v>note</x:v>
+        <x:v>region</x:v>
       </x:c>
       <x:c r="C31" s="41" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
+        <x:v>Clinical region category summarized only at cohort level.</x:v>
       </x:c>
       <x:c r="D31" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="26" t="str">
+      <x:c r="A32" s="49" t="str">
         <x:v>Fig_3</x:v>
       </x:c>
-      <x:c r="B32" s="27" t="str">
-        <x:v>panel</x:v>
-      </x:c>
-      <x:c r="C32" s="40" t="str">
-        <x:v>Panel identifier in the revised figure.</x:v>
-      </x:c>
-      <x:c r="D32" s="28" t="str">
+      <x:c r="B32" s="50" t="str">
+        <x:v>estimate</x:v>
+      </x:c>
+      <x:c r="C32" s="59" t="str">
+        <x:v>Released cohort-level point estimate.</x:v>
+      </x:c>
+      <x:c r="D32" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -1960,26 +1998,26 @@
         <x:v>Fig_3</x:v>
       </x:c>
       <x:c r="B33" s="15" t="str">
-        <x:v>metric</x:v>
+        <x:v>ci_low</x:v>
       </x:c>
       <x:c r="C33" s="41" t="str">
-        <x:v>Quantity summarized by the row.</x:v>
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D33" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="26" t="str">
+      <x:c r="A34" s="49" t="str">
         <x:v>Fig_3</x:v>
       </x:c>
-      <x:c r="B34" s="27" t="str">
-        <x:v>region</x:v>
-      </x:c>
-      <x:c r="C34" s="40" t="str">
-        <x:v>Clinical region category summarized only at cohort level.</x:v>
-      </x:c>
-      <x:c r="D34" s="28" t="str">
+      <x:c r="B34" s="50" t="str">
+        <x:v>ci_high</x:v>
+      </x:c>
+      <x:c r="C34" s="59" t="str">
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D34" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -1988,26 +2026,26 @@
         <x:v>Fig_3</x:v>
       </x:c>
       <x:c r="B35" s="15" t="str">
-        <x:v>estimate</x:v>
+        <x:v>adjusted_p</x:v>
       </x:c>
       <x:c r="C35" s="41" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
+        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
       </x:c>
       <x:c r="D35" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
-      <x:c r="A36" s="26" t="str">
+      <x:c r="A36" s="49" t="str">
         <x:v>Fig_3</x:v>
       </x:c>
-      <x:c r="B36" s="27" t="str">
-        <x:v>ci_low</x:v>
-      </x:c>
-      <x:c r="C36" s="40" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D36" s="28" t="str">
+      <x:c r="B36" s="50" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="C36" s="59" t="str">
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+      </x:c>
+      <x:c r="D36" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2016,82 +2054,82 @@
         <x:v>Fig_3</x:v>
       </x:c>
       <x:c r="B37" s="15" t="str">
-        <x:v>ci_high</x:v>
+        <x:v>analysis_unit</x:v>
       </x:c>
       <x:c r="C37" s="41" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Unit represented by the released row.</x:v>
       </x:c>
       <x:c r="D37" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
-      <x:c r="A38" s="26" t="str">
+      <x:c r="A38" s="49" t="str">
         <x:v>Fig_3</x:v>
       </x:c>
-      <x:c r="B38" s="27" t="str">
-        <x:v>adjusted_p</x:v>
-      </x:c>
-      <x:c r="C38" s="40" t="str">
-        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
-      </x:c>
-      <x:c r="D38" s="28" t="str">
+      <x:c r="B38" s="50" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C38" s="59" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D38" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="14" t="str">
-        <x:v>Fig_3</x:v>
+        <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B39" s="15" t="str">
-        <x:v>n</x:v>
+        <x:v>panel</x:v>
       </x:c>
       <x:c r="C39" s="41" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+        <x:v>Panel identifier in the revised figure.</x:v>
       </x:c>
       <x:c r="D39" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
-      <x:c r="A40" s="26" t="str">
-        <x:v>Fig_3</x:v>
-      </x:c>
-      <x:c r="B40" s="27" t="str">
-        <x:v>analysis_unit</x:v>
-      </x:c>
-      <x:c r="C40" s="40" t="str">
-        <x:v>Unit represented by the released row.</x:v>
-      </x:c>
-      <x:c r="D40" s="28" t="str">
+      <x:c r="A40" s="49" t="str">
+        <x:v>Fig_4</x:v>
+      </x:c>
+      <x:c r="B40" s="50" t="str">
+        <x:v>metric</x:v>
+      </x:c>
+      <x:c r="C40" s="59" t="str">
+        <x:v>Quantity summarized by the row.</x:v>
+      </x:c>
+      <x:c r="D40" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="14" t="str">
-        <x:v>Fig_3</x:v>
+        <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B41" s="15" t="str">
-        <x:v>note</x:v>
+        <x:v>stage</x:v>
       </x:c>
       <x:c r="C41" s="41" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
+        <x:v>Seizure stage in the aggregate contrast.</x:v>
       </x:c>
       <x:c r="D41" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
-      <x:c r="A42" s="26" t="str">
+      <x:c r="A42" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B42" s="27" t="str">
-        <x:v>panel</x:v>
-      </x:c>
-      <x:c r="C42" s="40" t="str">
-        <x:v>Panel identifier in the revised figure.</x:v>
-      </x:c>
-      <x:c r="D42" s="28" t="str">
+      <x:c r="B42" s="50" t="str">
+        <x:v>contrast</x:v>
+      </x:c>
+      <x:c r="C42" s="59" t="str">
+        <x:v>Direction and terms of the reported comparison.</x:v>
+      </x:c>
+      <x:c r="D42" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2100,26 +2138,26 @@
         <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B43" s="15" t="str">
-        <x:v>metric</x:v>
+        <x:v>estimate</x:v>
       </x:c>
       <x:c r="C43" s="41" t="str">
-        <x:v>Quantity summarized by the row.</x:v>
+        <x:v>Released cohort-level point estimate.</x:v>
       </x:c>
       <x:c r="D43" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
-      <x:c r="A44" s="26" t="str">
+      <x:c r="A44" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B44" s="27" t="str">
-        <x:v>stage</x:v>
-      </x:c>
-      <x:c r="C44" s="40" t="str">
-        <x:v>Seizure stage in the aggregate contrast.</x:v>
-      </x:c>
-      <x:c r="D44" s="28" t="str">
+      <x:c r="B44" s="50" t="str">
+        <x:v>median</x:v>
+      </x:c>
+      <x:c r="C44" s="59" t="str">
+        <x:v>Cohort median.</x:v>
+      </x:c>
+      <x:c r="D44" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2128,26 +2166,26 @@
         <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B45" s="15" t="str">
-        <x:v>contrast</x:v>
+        <x:v>ci_low</x:v>
       </x:c>
       <x:c r="C45" s="41" t="str">
-        <x:v>Direction and terms of the reported comparison.</x:v>
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D45" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
-      <x:c r="A46" s="26" t="str">
+      <x:c r="A46" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B46" s="27" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="C46" s="40" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
-      </x:c>
-      <x:c r="D46" s="28" t="str">
+      <x:c r="B46" s="50" t="str">
+        <x:v>ci_high</x:v>
+      </x:c>
+      <x:c r="C46" s="59" t="str">
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D46" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2156,26 +2194,26 @@
         <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B47" s="15" t="str">
-        <x:v>median</x:v>
+        <x:v>p_value</x:v>
       </x:c>
       <x:c r="C47" s="41" t="str">
-        <x:v>Cohort median.</x:v>
+        <x:v>Two-sided exact P value where applicable.</x:v>
       </x:c>
       <x:c r="D47" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
-      <x:c r="A48" s="26" t="str">
+      <x:c r="A48" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B48" s="27" t="str">
-        <x:v>ci_low</x:v>
-      </x:c>
-      <x:c r="C48" s="40" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D48" s="28" t="str">
+      <x:c r="B48" s="50" t="str">
+        <x:v>adjusted_p</x:v>
+      </x:c>
+      <x:c r="C48" s="59" t="str">
+        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
+      </x:c>
+      <x:c r="D48" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2184,26 +2222,26 @@
         <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B49" s="15" t="str">
-        <x:v>ci_high</x:v>
+        <x:v>n</x:v>
       </x:c>
       <x:c r="C49" s="41" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
       </x:c>
       <x:c r="D49" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
-      <x:c r="A50" s="26" t="str">
+      <x:c r="A50" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B50" s="27" t="str">
-        <x:v>p_value</x:v>
-      </x:c>
-      <x:c r="C50" s="40" t="str">
-        <x:v>Two-sided exact P value where applicable.</x:v>
-      </x:c>
-      <x:c r="D50" s="28" t="str">
+      <x:c r="B50" s="50" t="str">
+        <x:v>n_positive</x:v>
+      </x:c>
+      <x:c r="C50" s="59" t="str">
+        <x:v>Count of positive paired effects.</x:v>
+      </x:c>
+      <x:c r="D50" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2212,26 +2250,26 @@
         <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B51" s="15" t="str">
-        <x:v>adjusted_p</x:v>
+        <x:v>n_negative</x:v>
       </x:c>
       <x:c r="C51" s="41" t="str">
-        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
+        <x:v>Count of negative paired effects.</x:v>
       </x:c>
       <x:c r="D51" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
-      <x:c r="A52" s="26" t="str">
+      <x:c r="A52" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B52" s="27" t="str">
-        <x:v>n</x:v>
-      </x:c>
-      <x:c r="C52" s="40" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
-      </x:c>
-      <x:c r="D52" s="28" t="str">
+      <x:c r="B52" s="50" t="str">
+        <x:v>n_zero</x:v>
+      </x:c>
+      <x:c r="C52" s="59" t="str">
+        <x:v>Count of zero paired effects.</x:v>
+      </x:c>
+      <x:c r="D52" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2240,82 +2278,82 @@
         <x:v>Fig_4</x:v>
       </x:c>
       <x:c r="B53" s="15" t="str">
-        <x:v>n_positive</x:v>
+        <x:v>analysis_unit</x:v>
       </x:c>
       <x:c r="C53" s="41" t="str">
-        <x:v>Count of positive paired effects.</x:v>
+        <x:v>Unit represented by the released row.</x:v>
       </x:c>
       <x:c r="D53" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
-      <x:c r="A54" s="26" t="str">
+      <x:c r="A54" s="49" t="str">
         <x:v>Fig_4</x:v>
       </x:c>
-      <x:c r="B54" s="27" t="str">
-        <x:v>n_negative</x:v>
-      </x:c>
-      <x:c r="C54" s="40" t="str">
-        <x:v>Count of negative paired effects.</x:v>
-      </x:c>
-      <x:c r="D54" s="28" t="str">
+      <x:c r="B54" s="50" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C54" s="59" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D54" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="14" t="str">
-        <x:v>Fig_4</x:v>
+        <x:v>Fig_5</x:v>
       </x:c>
       <x:c r="B55" s="15" t="str">
-        <x:v>n_zero</x:v>
+        <x:v>panel</x:v>
       </x:c>
       <x:c r="C55" s="41" t="str">
-        <x:v>Count of zero paired effects.</x:v>
+        <x:v>Panel identifier in the revised figure.</x:v>
       </x:c>
       <x:c r="D55" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
-      <x:c r="A56" s="26" t="str">
-        <x:v>Fig_4</x:v>
-      </x:c>
-      <x:c r="B56" s="27" t="str">
-        <x:v>analysis_unit</x:v>
-      </x:c>
-      <x:c r="C56" s="40" t="str">
-        <x:v>Unit represented by the released row.</x:v>
-      </x:c>
-      <x:c r="D56" s="28" t="str">
+      <x:c r="A56" s="49" t="str">
+        <x:v>Fig_5</x:v>
+      </x:c>
+      <x:c r="B56" s="50" t="str">
+        <x:v>metric</x:v>
+      </x:c>
+      <x:c r="C56" s="59" t="str">
+        <x:v>Quantity summarized by the row.</x:v>
+      </x:c>
+      <x:c r="D56" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="14" t="str">
-        <x:v>Fig_4</x:v>
+        <x:v>Fig_5</x:v>
       </x:c>
       <x:c r="B57" s="15" t="str">
-        <x:v>note</x:v>
+        <x:v>series</x:v>
       </x:c>
       <x:c r="C57" s="41" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
+        <x:v>Method, configuration, or stage represented by the row.</x:v>
       </x:c>
       <x:c r="D57" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
-      <x:c r="A58" s="26" t="str">
+      <x:c r="A58" s="49" t="str">
         <x:v>Fig_5</x:v>
       </x:c>
-      <x:c r="B58" s="27" t="str">
-        <x:v>panel</x:v>
-      </x:c>
-      <x:c r="C58" s="40" t="str">
-        <x:v>Panel identifier in the revised figure.</x:v>
-      </x:c>
-      <x:c r="D58" s="28" t="str">
+      <x:c r="B58" s="50" t="str">
+        <x:v>contrast</x:v>
+      </x:c>
+      <x:c r="C58" s="59" t="str">
+        <x:v>Direction and terms of the reported comparison.</x:v>
+      </x:c>
+      <x:c r="D58" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2324,26 +2362,26 @@
         <x:v>Fig_5</x:v>
       </x:c>
       <x:c r="B59" s="15" t="str">
-        <x:v>metric</x:v>
+        <x:v>estimate</x:v>
       </x:c>
       <x:c r="C59" s="41" t="str">
-        <x:v>Quantity summarized by the row.</x:v>
+        <x:v>Released cohort-level point estimate.</x:v>
       </x:c>
       <x:c r="D59" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
-      <x:c r="A60" s="26" t="str">
+      <x:c r="A60" s="49" t="str">
         <x:v>Fig_5</x:v>
       </x:c>
-      <x:c r="B60" s="27" t="str">
-        <x:v>series</x:v>
-      </x:c>
-      <x:c r="C60" s="40" t="str">
-        <x:v>Method, configuration, or stage represented by the row.</x:v>
-      </x:c>
-      <x:c r="D60" s="28" t="str">
+      <x:c r="B60" s="50" t="str">
+        <x:v>ci_low</x:v>
+      </x:c>
+      <x:c r="C60" s="59" t="str">
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D60" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2352,26 +2390,26 @@
         <x:v>Fig_5</x:v>
       </x:c>
       <x:c r="B61" s="15" t="str">
-        <x:v>contrast</x:v>
+        <x:v>ci_high</x:v>
       </x:c>
       <x:c r="C61" s="41" t="str">
-        <x:v>Direction and terms of the reported comparison.</x:v>
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D61" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
-      <x:c r="A62" s="26" t="str">
+      <x:c r="A62" s="49" t="str">
         <x:v>Fig_5</x:v>
       </x:c>
-      <x:c r="B62" s="27" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="C62" s="40" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
-      </x:c>
-      <x:c r="D62" s="28" t="str">
+      <x:c r="B62" s="50" t="str">
+        <x:v>p_value</x:v>
+      </x:c>
+      <x:c r="C62" s="59" t="str">
+        <x:v>Two-sided exact P value where applicable.</x:v>
+      </x:c>
+      <x:c r="D62" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2380,26 +2418,26 @@
         <x:v>Fig_5</x:v>
       </x:c>
       <x:c r="B63" s="15" t="str">
-        <x:v>ci_low</x:v>
+        <x:v>adjusted_p</x:v>
       </x:c>
       <x:c r="C63" s="41" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
       </x:c>
       <x:c r="D63" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
-      <x:c r="A64" s="26" t="str">
+      <x:c r="A64" s="49" t="str">
         <x:v>Fig_5</x:v>
       </x:c>
-      <x:c r="B64" s="27" t="str">
-        <x:v>ci_high</x:v>
-      </x:c>
-      <x:c r="C64" s="40" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D64" s="28" t="str">
+      <x:c r="B64" s="50" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="C64" s="59" t="str">
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+      </x:c>
+      <x:c r="D64" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2408,82 +2446,82 @@
         <x:v>Fig_5</x:v>
       </x:c>
       <x:c r="B65" s="15" t="str">
-        <x:v>p_value</x:v>
+        <x:v>analysis_unit</x:v>
       </x:c>
       <x:c r="C65" s="41" t="str">
-        <x:v>Two-sided exact P value where applicable.</x:v>
+        <x:v>Unit represented by the released row.</x:v>
       </x:c>
       <x:c r="D65" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
-      <x:c r="A66" s="26" t="str">
+      <x:c r="A66" s="49" t="str">
         <x:v>Fig_5</x:v>
       </x:c>
-      <x:c r="B66" s="27" t="str">
-        <x:v>adjusted_p</x:v>
-      </x:c>
-      <x:c r="C66" s="40" t="str">
-        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
-      </x:c>
-      <x:c r="D66" s="28" t="str">
+      <x:c r="B66" s="50" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C66" s="59" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D66" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="14" t="str">
-        <x:v>Fig_5</x:v>
+        <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B67" s="15" t="str">
-        <x:v>n</x:v>
+        <x:v>panel</x:v>
       </x:c>
       <x:c r="C67" s="41" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+        <x:v>Panel identifier in the revised figure.</x:v>
       </x:c>
       <x:c r="D67" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
-      <x:c r="A68" s="26" t="str">
-        <x:v>Fig_5</x:v>
-      </x:c>
-      <x:c r="B68" s="27" t="str">
-        <x:v>analysis_unit</x:v>
-      </x:c>
-      <x:c r="C68" s="40" t="str">
-        <x:v>Unit represented by the released row.</x:v>
-      </x:c>
-      <x:c r="D68" s="28" t="str">
+      <x:c r="A68" s="49" t="str">
+        <x:v>Fig_6</x:v>
+      </x:c>
+      <x:c r="B68" s="50" t="str">
+        <x:v>group</x:v>
+      </x:c>
+      <x:c r="C68" s="59" t="str">
+        <x:v>Sensitivity or strategy family.</x:v>
+      </x:c>
+      <x:c r="D68" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="14" t="str">
-        <x:v>Fig_5</x:v>
+        <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B69" s="15" t="str">
-        <x:v>note</x:v>
+        <x:v>label</x:v>
       </x:c>
       <x:c r="C69" s="41" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
+        <x:v>Display label for a public aggregate setting.</x:v>
       </x:c>
       <x:c r="D69" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
-      <x:c r="A70" s="26" t="str">
+      <x:c r="A70" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B70" s="27" t="str">
-        <x:v>panel</x:v>
-      </x:c>
-      <x:c r="C70" s="40" t="str">
-        <x:v>Panel identifier in the revised figure.</x:v>
-      </x:c>
-      <x:c r="D70" s="28" t="str">
+      <x:c r="B70" s="50" t="str">
+        <x:v>metric</x:v>
+      </x:c>
+      <x:c r="C70" s="59" t="str">
+        <x:v>Quantity summarized by the row.</x:v>
+      </x:c>
+      <x:c r="D70" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2492,26 +2530,26 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B71" s="15" t="str">
-        <x:v>group</x:v>
+        <x:v>estimate</x:v>
       </x:c>
       <x:c r="C71" s="41" t="str">
-        <x:v>Sensitivity or strategy family.</x:v>
+        <x:v>Released cohort-level point estimate.</x:v>
       </x:c>
       <x:c r="D71" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
-      <x:c r="A72" s="26" t="str">
+      <x:c r="A72" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B72" s="27" t="str">
-        <x:v>label</x:v>
-      </x:c>
-      <x:c r="C72" s="40" t="str">
-        <x:v>Display label for a public aggregate setting.</x:v>
-      </x:c>
-      <x:c r="D72" s="28" t="str">
+      <x:c r="B72" s="50" t="str">
+        <x:v>ci_low</x:v>
+      </x:c>
+      <x:c r="C72" s="59" t="str">
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D72" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2520,26 +2558,26 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B73" s="15" t="str">
-        <x:v>metric</x:v>
+        <x:v>ci_high</x:v>
       </x:c>
       <x:c r="C73" s="41" t="str">
-        <x:v>Quantity summarized by the row.</x:v>
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D73" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
-      <x:c r="A74" s="26" t="str">
+      <x:c r="A74" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B74" s="27" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="C74" s="40" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
-      </x:c>
-      <x:c r="D74" s="28" t="str">
+      <x:c r="B74" s="50" t="str">
+        <x:v>n</x:v>
+      </x:c>
+      <x:c r="C74" s="59" t="str">
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+      </x:c>
+      <x:c r="D74" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2548,26 +2586,26 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B75" s="15" t="str">
-        <x:v>ci_low</x:v>
+        <x:v>is_reference</x:v>
       </x:c>
       <x:c r="C75" s="41" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Whether the row is the frozen sensitivity reference or deterministic path reference.</x:v>
       </x:c>
       <x:c r="D75" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
-      <x:c r="A76" s="26" t="str">
+      <x:c r="A76" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B76" s="27" t="str">
-        <x:v>ci_high</x:v>
-      </x:c>
-      <x:c r="C76" s="40" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D76" s="28" t="str">
+      <x:c r="B76" s="50" t="str">
+        <x:v>candidate_metric</x:v>
+      </x:c>
+      <x:c r="C76" s="59" t="str">
+        <x:v>Pairwise candidate metric; MSC does not denote COC.</x:v>
+      </x:c>
+      <x:c r="D76" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2576,26 +2614,26 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B77" s="15" t="str">
-        <x:v>n</x:v>
+        <x:v>pair_retained_fraction</x:v>
       </x:c>
       <x:c r="C77" s="41" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
+        <x:v>Exact pair fraction used only in sensitivity analysis.</x:v>
       </x:c>
       <x:c r="D77" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
-      <x:c r="A78" s="26" t="str">
+      <x:c r="A78" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B78" s="27" t="str">
-        <x:v>is_reference</x:v>
-      </x:c>
-      <x:c r="C78" s="40" t="str">
-        <x:v>Whether the row is the frozen sensitivity reference or deterministic path reference.</x:v>
-      </x:c>
-      <x:c r="D78" s="28" t="str">
+      <x:c r="B78" s="50" t="str">
+        <x:v>hyper_mode</x:v>
+      </x:c>
+      <x:c r="C78" s="59" t="str">
+        <x:v>Higher-order weighting mode in the sensitivity grid.</x:v>
+      </x:c>
+      <x:c r="D78" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2604,26 +2642,26 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B79" s="15" t="str">
-        <x:v>candidate_metric</x:v>
+        <x:v>window_sec</x:v>
       </x:c>
       <x:c r="C79" s="41" t="str">
-        <x:v>Pairwise candidate metric; MSC does not denote COC.</x:v>
+        <x:v>Window length in seconds.</x:v>
       </x:c>
       <x:c r="D79" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
-      <x:c r="A80" s="26" t="str">
+      <x:c r="A80" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B80" s="27" t="str">
-        <x:v>pair_retained_fraction</x:v>
-      </x:c>
-      <x:c r="C80" s="40" t="str">
-        <x:v>Exact pair fraction used only in sensitivity analysis.</x:v>
-      </x:c>
-      <x:c r="D80" s="28" t="str">
+      <x:c r="B80" s="50" t="str">
+        <x:v>step_sec</x:v>
+      </x:c>
+      <x:c r="C80" s="59" t="str">
+        <x:v>Window step in seconds.</x:v>
+      </x:c>
+      <x:c r="D80" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2632,26 +2670,26 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B81" s="15" t="str">
-        <x:v>hyper_mode</x:v>
+        <x:v>alpha</x:v>
       </x:c>
       <x:c r="C81" s="41" t="str">
-        <x:v>Higher-order weighting mode in the sensitivity grid.</x:v>
+        <x:v>Adjacent-window temporal fusion weight.</x:v>
       </x:c>
       <x:c r="D81" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
-      <x:c r="A82" s="26" t="str">
+      <x:c r="A82" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B82" s="27" t="str">
-        <x:v>window_sec</x:v>
-      </x:c>
-      <x:c r="C82" s="40" t="str">
-        <x:v>Window length in seconds.</x:v>
-      </x:c>
-      <x:c r="D82" s="28" t="str">
+      <x:c r="B82" s="50" t="str">
+        <x:v>bandwidth_multiplier</x:v>
+      </x:c>
+      <x:c r="C82" s="59" t="str">
+        <x:v>Multiplier applied to the MAD Gaussian-kernel bandwidth.</x:v>
+      </x:c>
+      <x:c r="D82" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2660,82 +2698,82 @@
         <x:v>Fig_6</x:v>
       </x:c>
       <x:c r="B83" s="15" t="str">
-        <x:v>step_sec</x:v>
+        <x:v>top_fraction</x:v>
       </x:c>
       <x:c r="C83" s="41" t="str">
-        <x:v>Window step in seconds.</x:v>
+        <x:v>Candidate fraction used by the jump strategy.</x:v>
       </x:c>
       <x:c r="D83" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
-      <x:c r="A84" s="26" t="str">
+      <x:c r="A84" s="49" t="str">
         <x:v>Fig_6</x:v>
       </x:c>
-      <x:c r="B84" s="27" t="str">
-        <x:v>alpha</x:v>
-      </x:c>
-      <x:c r="C84" s="40" t="str">
-        <x:v>Adjacent-window temporal fusion weight.</x:v>
-      </x:c>
-      <x:c r="D84" s="28" t="str">
+      <x:c r="B84" s="50" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C84" s="59" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D84" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
       <x:c r="A85" s="14" t="str">
-        <x:v>Fig_6</x:v>
+        <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B85" s="15" t="str">
-        <x:v>bandwidth_multiplier</x:v>
+        <x:v>configuration</x:v>
       </x:c>
       <x:c r="C85" s="41" t="str">
-        <x:v>Multiplier applied to the MAD Gaussian-kernel bandwidth.</x:v>
+        <x:v>Public sensitivity configuration name without participant information.</x:v>
       </x:c>
       <x:c r="D85" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
-      <x:c r="A86" s="26" t="str">
-        <x:v>Fig_6</x:v>
-      </x:c>
-      <x:c r="B86" s="27" t="str">
-        <x:v>top_fraction</x:v>
-      </x:c>
-      <x:c r="C86" s="40" t="str">
-        <x:v>Candidate fraction used by the jump strategy.</x:v>
-      </x:c>
-      <x:c r="D86" s="28" t="str">
+      <x:c r="A86" s="49" t="str">
+        <x:v>Supp_Fig_S1</x:v>
+      </x:c>
+      <x:c r="B86" s="50" t="str">
+        <x:v>family</x:v>
+      </x:c>
+      <x:c r="C86" s="59" t="str">
+        <x:v>Sensitivity family.</x:v>
+      </x:c>
+      <x:c r="D86" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
       <x:c r="A87" s="14" t="str">
-        <x:v>Fig_6</x:v>
+        <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B87" s="15" t="str">
-        <x:v>note</x:v>
+        <x:v>label</x:v>
       </x:c>
       <x:c r="C87" s="41" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
+        <x:v>Display label for a public aggregate setting.</x:v>
       </x:c>
       <x:c r="D87" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
-      <x:c r="A88" s="26" t="str">
+      <x:c r="A88" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B88" s="27" t="str">
-        <x:v>configuration</x:v>
-      </x:c>
-      <x:c r="C88" s="40" t="str">
-        <x:v>Public sensitivity configuration name without participant information.</x:v>
-      </x:c>
-      <x:c r="D88" s="28" t="str">
+      <x:c r="B88" s="50" t="str">
+        <x:v>candidate_metric</x:v>
+      </x:c>
+      <x:c r="C88" s="59" t="str">
+        <x:v>Pairwise candidate metric; MSC does not denote COC.</x:v>
+      </x:c>
+      <x:c r="D88" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2744,26 +2782,26 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B89" s="15" t="str">
-        <x:v>family</x:v>
+        <x:v>pair_retained_fraction</x:v>
       </x:c>
       <x:c r="C89" s="41" t="str">
-        <x:v>Sensitivity family.</x:v>
+        <x:v>Exact pair fraction used only in sensitivity analysis.</x:v>
       </x:c>
       <x:c r="D89" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
-      <x:c r="A90" s="26" t="str">
+      <x:c r="A90" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B90" s="27" t="str">
-        <x:v>label</x:v>
-      </x:c>
-      <x:c r="C90" s="40" t="str">
-        <x:v>Display label for a public aggregate setting.</x:v>
-      </x:c>
-      <x:c r="D90" s="28" t="str">
+      <x:c r="B90" s="50" t="str">
+        <x:v>hyper_mode</x:v>
+      </x:c>
+      <x:c r="C90" s="59" t="str">
+        <x:v>Higher-order weighting mode in the sensitivity grid.</x:v>
+      </x:c>
+      <x:c r="D90" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2772,26 +2810,26 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B91" s="15" t="str">
-        <x:v>candidate_metric</x:v>
+        <x:v>window_sec</x:v>
       </x:c>
       <x:c r="C91" s="41" t="str">
-        <x:v>Pairwise candidate metric; MSC does not denote COC.</x:v>
+        <x:v>Window length in seconds.</x:v>
       </x:c>
       <x:c r="D91" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
-      <x:c r="A92" s="26" t="str">
+      <x:c r="A92" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B92" s="27" t="str">
-        <x:v>pair_retained_fraction</x:v>
-      </x:c>
-      <x:c r="C92" s="40" t="str">
-        <x:v>Exact pair fraction used only in sensitivity analysis.</x:v>
-      </x:c>
-      <x:c r="D92" s="28" t="str">
+      <x:c r="B92" s="50" t="str">
+        <x:v>step_sec</x:v>
+      </x:c>
+      <x:c r="C92" s="59" t="str">
+        <x:v>Window step in seconds.</x:v>
+      </x:c>
+      <x:c r="D92" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2800,26 +2838,26 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B93" s="15" t="str">
-        <x:v>hyper_mode</x:v>
+        <x:v>alpha</x:v>
       </x:c>
       <x:c r="C93" s="41" t="str">
-        <x:v>Higher-order weighting mode in the sensitivity grid.</x:v>
+        <x:v>Adjacent-window temporal fusion weight.</x:v>
       </x:c>
       <x:c r="D93" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="15" hidden="0" customHeight="1">
-      <x:c r="A94" s="26" t="str">
+      <x:c r="A94" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B94" s="27" t="str">
-        <x:v>window_sec</x:v>
-      </x:c>
-      <x:c r="C94" s="40" t="str">
-        <x:v>Window length in seconds.</x:v>
-      </x:c>
-      <x:c r="D94" s="28" t="str">
+      <x:c r="B94" s="50" t="str">
+        <x:v>bandwidth_multiplier</x:v>
+      </x:c>
+      <x:c r="C94" s="59" t="str">
+        <x:v>Multiplier applied to the MAD Gaussian-kernel bandwidth.</x:v>
+      </x:c>
+      <x:c r="D94" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2828,26 +2866,26 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B95" s="15" t="str">
-        <x:v>step_sec</x:v>
+        <x:v>estimate</x:v>
       </x:c>
       <x:c r="C95" s="41" t="str">
-        <x:v>Window step in seconds.</x:v>
+        <x:v>Released cohort-level point estimate.</x:v>
       </x:c>
       <x:c r="D95" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="96" ht="15" hidden="0" customHeight="1">
-      <x:c r="A96" s="26" t="str">
+      <x:c r="A96" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B96" s="27" t="str">
-        <x:v>alpha</x:v>
-      </x:c>
-      <x:c r="C96" s="40" t="str">
-        <x:v>Adjacent-window temporal fusion weight.</x:v>
-      </x:c>
-      <x:c r="D96" s="28" t="str">
+      <x:c r="B96" s="50" t="str">
+        <x:v>median</x:v>
+      </x:c>
+      <x:c r="C96" s="59" t="str">
+        <x:v>Cohort median.</x:v>
+      </x:c>
+      <x:c r="D96" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2856,26 +2894,26 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B97" s="15" t="str">
-        <x:v>bandwidth_multiplier</x:v>
+        <x:v>ci_low</x:v>
       </x:c>
       <x:c r="C97" s="41" t="str">
-        <x:v>Multiplier applied to the MAD Gaussian-kernel bandwidth.</x:v>
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D97" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="98" ht="15" hidden="0" customHeight="1">
-      <x:c r="A98" s="26" t="str">
+      <x:c r="A98" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B98" s="27" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="C98" s="40" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
-      </x:c>
-      <x:c r="D98" s="28" t="str">
+      <x:c r="B98" s="50" t="str">
+        <x:v>ci_high</x:v>
+      </x:c>
+      <x:c r="C98" s="59" t="str">
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D98" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2884,26 +2922,26 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B99" s="15" t="str">
-        <x:v>median</x:v>
+        <x:v>n</x:v>
       </x:c>
       <x:c r="C99" s="41" t="str">
-        <x:v>Cohort median.</x:v>
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
       </x:c>
       <x:c r="D99" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="100" ht="15" hidden="0" customHeight="1">
-      <x:c r="A100" s="26" t="str">
+      <x:c r="A100" s="49" t="str">
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
-      <x:c r="B100" s="27" t="str">
-        <x:v>ci_low</x:v>
-      </x:c>
-      <x:c r="C100" s="40" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D100" s="28" t="str">
+      <x:c r="B100" s="50" t="str">
+        <x:v>is_reference</x:v>
+      </x:c>
+      <x:c r="C100" s="59" t="str">
+        <x:v>Whether the row is the frozen sensitivity reference or deterministic path reference.</x:v>
+      </x:c>
+      <x:c r="D100" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2912,54 +2950,54 @@
         <x:v>Supp_Fig_S1</x:v>
       </x:c>
       <x:c r="B101" s="15" t="str">
-        <x:v>ci_high</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C101" s="41" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Interpretive or privacy note.</x:v>
       </x:c>
       <x:c r="D101" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="15" hidden="0" customHeight="1">
-      <x:c r="A102" s="26" t="str">
-        <x:v>Supp_Fig_S1</x:v>
-      </x:c>
-      <x:c r="B102" s="27" t="str">
-        <x:v>n</x:v>
-      </x:c>
-      <x:c r="C102" s="40" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
-      </x:c>
-      <x:c r="D102" s="28" t="str">
+      <x:c r="A102" s="49" t="str">
+        <x:v>Supp_Fig_S2</x:v>
+      </x:c>
+      <x:c r="B102" s="50" t="str">
+        <x:v>panel</x:v>
+      </x:c>
+      <x:c r="C102" s="59" t="str">
+        <x:v>Panel identifier in the revised figure.</x:v>
+      </x:c>
+      <x:c r="D102" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="103" ht="15" hidden="0" customHeight="1">
       <x:c r="A103" s="14" t="str">
-        <x:v>Supp_Fig_S1</x:v>
+        <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B103" s="15" t="str">
-        <x:v>is_reference</x:v>
+        <x:v>analysis</x:v>
       </x:c>
       <x:c r="C103" s="41" t="str">
-        <x:v>Whether the row is the frozen sensitivity reference or deterministic path reference.</x:v>
+        <x:v>Null or boundary analysis.</x:v>
       </x:c>
       <x:c r="D103" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="104" ht="15" hidden="0" customHeight="1">
-      <x:c r="A104" s="26" t="str">
-        <x:v>Supp_Fig_S1</x:v>
-      </x:c>
-      <x:c r="B104" s="27" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="C104" s="40" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
-      </x:c>
-      <x:c r="D104" s="28" t="str">
+      <x:c r="A104" s="49" t="str">
+        <x:v>Supp_Fig_S2</x:v>
+      </x:c>
+      <x:c r="B104" s="50" t="str">
+        <x:v>target</x:v>
+      </x:c>
+      <x:c r="C104" s="59" t="str">
+        <x:v>Aggregate target category.</x:v>
+      </x:c>
+      <x:c r="D104" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2968,26 +3006,26 @@
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B105" s="15" t="str">
-        <x:v>panel</x:v>
+        <x:v>contrast</x:v>
       </x:c>
       <x:c r="C105" s="41" t="str">
-        <x:v>Panel identifier in the revised figure.</x:v>
+        <x:v>Direction and terms of the reported comparison.</x:v>
       </x:c>
       <x:c r="D105" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="106" ht="15" hidden="0" customHeight="1">
-      <x:c r="A106" s="26" t="str">
+      <x:c r="A106" s="49" t="str">
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
-      <x:c r="B106" s="27" t="str">
-        <x:v>analysis</x:v>
-      </x:c>
-      <x:c r="C106" s="40" t="str">
-        <x:v>Null or boundary analysis.</x:v>
-      </x:c>
-      <x:c r="D106" s="28" t="str">
+      <x:c r="B106" s="50" t="str">
+        <x:v>estimate</x:v>
+      </x:c>
+      <x:c r="C106" s="59" t="str">
+        <x:v>Released cohort-level point estimate.</x:v>
+      </x:c>
+      <x:c r="D106" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -2996,26 +3034,26 @@
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B107" s="15" t="str">
-        <x:v>target</x:v>
+        <x:v>ci_low</x:v>
       </x:c>
       <x:c r="C107" s="41" t="str">
-        <x:v>Aggregate target category.</x:v>
+        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
       </x:c>
       <x:c r="D107" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="108" ht="15" hidden="0" customHeight="1">
-      <x:c r="A108" s="26" t="str">
+      <x:c r="A108" s="49" t="str">
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
-      <x:c r="B108" s="27" t="str">
-        <x:v>contrast</x:v>
-      </x:c>
-      <x:c r="C108" s="40" t="str">
-        <x:v>Direction and terms of the reported comparison.</x:v>
-      </x:c>
-      <x:c r="D108" s="28" t="str">
+      <x:c r="B108" s="50" t="str">
+        <x:v>ci_high</x:v>
+      </x:c>
+      <x:c r="C108" s="59" t="str">
+        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+      </x:c>
+      <x:c r="D108" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -3024,26 +3062,26 @@
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B109" s="15" t="str">
-        <x:v>estimate</x:v>
+        <x:v>p_value</x:v>
       </x:c>
       <x:c r="C109" s="41" t="str">
-        <x:v>Released cohort-level point estimate.</x:v>
+        <x:v>Two-sided exact P value where applicable.</x:v>
       </x:c>
       <x:c r="D109" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="15" hidden="0" customHeight="1">
-      <x:c r="A110" s="26" t="str">
+      <x:c r="A110" s="49" t="str">
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
-      <x:c r="B110" s="27" t="str">
-        <x:v>ci_low</x:v>
-      </x:c>
-      <x:c r="C110" s="40" t="str">
-        <x:v>Lower bound of the participant-bootstrap 95% confidence interval.</x:v>
-      </x:c>
-      <x:c r="D110" s="28" t="str">
+      <x:c r="B110" s="50" t="str">
+        <x:v>adjusted_p</x:v>
+      </x:c>
+      <x:c r="C110" s="59" t="str">
+        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
+      </x:c>
+      <x:c r="D110" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -3052,26 +3090,26 @@
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B111" s="15" t="str">
-        <x:v>ci_high</x:v>
+        <x:v>n</x:v>
       </x:c>
       <x:c r="C111" s="41" t="str">
-        <x:v>Upper bound of the participant-bootstrap 95% confidence interval.</x:v>
+        <x:v>Number of independent participants contributing to the aggregate.</x:v>
       </x:c>
       <x:c r="D111" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="112" ht="15" hidden="0" customHeight="1">
-      <x:c r="A112" s="26" t="str">
+      <x:c r="A112" s="49" t="str">
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
-      <x:c r="B112" s="27" t="str">
-        <x:v>p_value</x:v>
-      </x:c>
-      <x:c r="C112" s="40" t="str">
-        <x:v>Two-sided exact P value where applicable.</x:v>
-      </x:c>
-      <x:c r="D112" s="28" t="str">
+      <x:c r="B112" s="50" t="str">
+        <x:v>n_positive</x:v>
+      </x:c>
+      <x:c r="C112" s="59" t="str">
+        <x:v>Count of positive paired effects.</x:v>
+      </x:c>
+      <x:c r="D112" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -3080,26 +3118,26 @@
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B113" s="15" t="str">
-        <x:v>adjusted_p</x:v>
+        <x:v>n_negative</x:v>
       </x:c>
       <x:c r="C113" s="41" t="str">
-        <x:v>Benjamini–Hochberg adjusted P value where applicable.</x:v>
+        <x:v>Count of negative paired effects.</x:v>
       </x:c>
       <x:c r="D113" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="114" ht="15" hidden="0" customHeight="1">
-      <x:c r="A114" s="26" t="str">
+      <x:c r="A114" s="49" t="str">
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
-      <x:c r="B114" s="27" t="str">
-        <x:v>n</x:v>
-      </x:c>
-      <x:c r="C114" s="40" t="str">
-        <x:v>Number of independent participants contributing to the aggregate.</x:v>
-      </x:c>
-      <x:c r="D114" s="28" t="str">
+      <x:c r="B114" s="50" t="str">
+        <x:v>n_zero</x:v>
+      </x:c>
+      <x:c r="C114" s="59" t="str">
+        <x:v>Count of zero paired effects.</x:v>
+      </x:c>
+      <x:c r="D114" s="51" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
@@ -3108,55 +3146,55 @@
         <x:v>Supp_Fig_S2</x:v>
       </x:c>
       <x:c r="B115" s="15" t="str">
-        <x:v>n_positive</x:v>
+        <x:v>note</x:v>
       </x:c>
       <x:c r="C115" s="41" t="str">
-        <x:v>Count of positive paired effects.</x:v>
+        <x:v>Interpretive or privacy note.</x:v>
       </x:c>
       <x:c r="D115" s="16" t="str">
         <x:v>cohort aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="116" ht="15" hidden="0" customHeight="1">
-      <x:c r="A116" s="26" t="str">
-        <x:v>Supp_Fig_S2</x:v>
-      </x:c>
-      <x:c r="B116" s="27" t="str">
-        <x:v>n_negative</x:v>
-      </x:c>
-      <x:c r="C116" s="40" t="str">
-        <x:v>Count of negative paired effects.</x:v>
-      </x:c>
-      <x:c r="D116" s="28" t="str">
-        <x:v>cohort aggregate</x:v>
+      <x:c r="A116" s="49" t="str">
+        <x:v>Numeric_Tests</x:v>
+      </x:c>
+      <x:c r="B116" s="50" t="str">
+        <x:v>test</x:v>
+      </x:c>
+      <x:c r="C116" s="59" t="str">
+        <x:v>Synthetic numerical test name.</x:v>
+      </x:c>
+      <x:c r="D116" s="51" t="str">
+        <x:v>synthetic</x:v>
       </x:c>
     </x:row>
     <x:row r="117" ht="15" hidden="0" customHeight="1">
       <x:c r="A117" s="14" t="str">
-        <x:v>Supp_Fig_S2</x:v>
+        <x:v>Numeric_Tests</x:v>
       </x:c>
       <x:c r="B117" s="15" t="str">
-        <x:v>n_zero</x:v>
+        <x:v>passed</x:v>
       </x:c>
       <x:c r="C117" s="41" t="str">
-        <x:v>Count of zero paired effects.</x:v>
+        <x:v>Whether the synthetic boundary test passed.</x:v>
       </x:c>
       <x:c r="D117" s="16" t="str">
-        <x:v>cohort aggregate</x:v>
+        <x:v>synthetic</x:v>
       </x:c>
     </x:row>
     <x:row r="118" ht="15" hidden="0" customHeight="1">
-      <x:c r="A118" s="26" t="str">
-        <x:v>Supp_Fig_S2</x:v>
-      </x:c>
-      <x:c r="B118" s="27" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="C118" s="40" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
-      </x:c>
-      <x:c r="D118" s="28" t="str">
-        <x:v>cohort aggregate</x:v>
+      <x:c r="A118" s="49" t="str">
+        <x:v>Numeric_Tests</x:v>
+      </x:c>
+      <x:c r="B118" s="50" t="str">
+        <x:v>diagnostic</x:v>
+      </x:c>
+      <x:c r="C118" s="59" t="str">
+        <x:v>Released numerical diagnostic for the test.</x:v>
+      </x:c>
+      <x:c r="D118" s="51" t="str">
+        <x:v>synthetic</x:v>
       </x:c>
     </x:row>
     <x:row r="119" ht="15" hidden="0" customHeight="1">
@@ -3164,82 +3202,82 @@
         <x:v>Numeric_Tests</x:v>
       </x:c>
       <x:c r="B119" s="15" t="str">
-        <x:v>test</x:v>
+        <x:v>data_level</x:v>
       </x:c>
       <x:c r="C119" s="41" t="str">
-        <x:v>Synthetic numerical test name.</x:v>
+        <x:v>Privacy/data level of the row.</x:v>
       </x:c>
       <x:c r="D119" s="16" t="str">
         <x:v>synthetic</x:v>
       </x:c>
     </x:row>
     <x:row r="120" ht="15" hidden="0" customHeight="1">
-      <x:c r="A120" s="26" t="str">
+      <x:c r="A120" s="49" t="str">
         <x:v>Numeric_Tests</x:v>
       </x:c>
-      <x:c r="B120" s="27" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="C120" s="40" t="str">
-        <x:v>Whether the synthetic boundary test passed.</x:v>
-      </x:c>
-      <x:c r="D120" s="28" t="str">
+      <x:c r="B120" s="50" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C120" s="59" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D120" s="51" t="str">
         <x:v>synthetic</x:v>
       </x:c>
     </x:row>
     <x:row r="121" ht="15" hidden="0" customHeight="1">
       <x:c r="A121" s="14" t="str">
-        <x:v>Numeric_Tests</x:v>
+        <x:v>Raw_Data_Summary</x:v>
       </x:c>
       <x:c r="B121" s="15" t="str">
-        <x:v>diagnostic</x:v>
+        <x:v>data_class</x:v>
       </x:c>
       <x:c r="C121" s="41" t="str">
-        <x:v>Released numerical diagnostic for the test.</x:v>
+        <x:v>Class of source or derived data.</x:v>
       </x:c>
       <x:c r="D121" s="16" t="str">
-        <x:v>synthetic</x:v>
+        <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="15" hidden="0" customHeight="1">
-      <x:c r="A122" s="26" t="str">
-        <x:v>Numeric_Tests</x:v>
-      </x:c>
-      <x:c r="B122" s="27" t="str">
-        <x:v>data_level</x:v>
-      </x:c>
-      <x:c r="C122" s="40" t="str">
-        <x:v>Privacy/data level of the row.</x:v>
-      </x:c>
-      <x:c r="D122" s="28" t="str">
-        <x:v>synthetic</x:v>
+      <x:c r="A122" s="49" t="str">
+        <x:v>Raw_Data_Summary</x:v>
+      </x:c>
+      <x:c r="B122" s="50" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C122" s="59" t="str">
+        <x:v>Public or restricted status.</x:v>
+      </x:c>
+      <x:c r="D122" s="51" t="str">
+        <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="123" ht="15" hidden="0" customHeight="1">
       <x:c r="A123" s="14" t="str">
-        <x:v>Numeric_Tests</x:v>
+        <x:v>Raw_Data_Summary</x:v>
       </x:c>
       <x:c r="B123" s="15" t="str">
-        <x:v>note</x:v>
+        <x:v>contents</x:v>
       </x:c>
       <x:c r="C123" s="41" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
+        <x:v>High-level contents without raw records.</x:v>
       </x:c>
       <x:c r="D123" s="16" t="str">
-        <x:v>synthetic</x:v>
+        <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="124" ht="15" hidden="0" customHeight="1">
-      <x:c r="A124" s="26" t="str">
+      <x:c r="A124" s="49" t="str">
         <x:v>Raw_Data_Summary</x:v>
       </x:c>
-      <x:c r="B124" s="27" t="str">
-        <x:v>data_class</x:v>
-      </x:c>
-      <x:c r="C124" s="40" t="str">
-        <x:v>Class of source or derived data.</x:v>
-      </x:c>
-      <x:c r="D124" s="28" t="str">
+      <x:c r="B124" s="50" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="C124" s="59" t="str">
+        <x:v>Granularity of the data class or metadata.</x:v>
+      </x:c>
+      <x:c r="D124" s="51" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
@@ -3248,26 +3286,26 @@
         <x:v>Raw_Data_Summary</x:v>
       </x:c>
       <x:c r="B125" s="15" t="str">
-        <x:v>status</x:v>
+        <x:v>public_representation</x:v>
       </x:c>
       <x:c r="C125" s="41" t="str">
-        <x:v>Public or restricted status.</x:v>
+        <x:v>Public aggregate representation.</x:v>
       </x:c>
       <x:c r="D125" s="16" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="126" ht="15" hidden="0" customHeight="1">
-      <x:c r="A126" s="26" t="str">
+      <x:c r="A126" s="49" t="str">
         <x:v>Raw_Data_Summary</x:v>
       </x:c>
-      <x:c r="B126" s="27" t="str">
-        <x:v>contents</x:v>
-      </x:c>
-      <x:c r="C126" s="40" t="str">
-        <x:v>High-level contents without raw records.</x:v>
-      </x:c>
-      <x:c r="D126" s="28" t="str">
+      <x:c r="B126" s="50" t="str">
+        <x:v>included</x:v>
+      </x:c>
+      <x:c r="C126" s="59" t="str">
+        <x:v>Whether records from the data class are included.</x:v>
+      </x:c>
+      <x:c r="D126" s="51" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
@@ -3276,145 +3314,121 @@
         <x:v>Raw_Data_Summary</x:v>
       </x:c>
       <x:c r="B127" s="15" t="str">
-        <x:v>level</x:v>
+        <x:v>access</x:v>
       </x:c>
       <x:c r="C127" s="41" t="str">
-        <x:v>Granularity of the data class or metadata.</x:v>
+        <x:v>Permitted access route.</x:v>
       </x:c>
       <x:c r="D127" s="16" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="128" ht="15" hidden="0" customHeight="1">
-      <x:c r="A128" s="26" t="str">
+      <x:c r="A128" s="49" t="str">
         <x:v>Raw_Data_Summary</x:v>
       </x:c>
-      <x:c r="B128" s="27" t="str">
-        <x:v>public_representation</x:v>
-      </x:c>
-      <x:c r="C128" s="40" t="str">
-        <x:v>Public aggregate representation.</x:v>
-      </x:c>
-      <x:c r="D128" s="28" t="str">
+      <x:c r="B128" s="50" t="str">
+        <x:v>privacy_rationale</x:v>
+      </x:c>
+      <x:c r="C128" s="59" t="str">
+        <x:v>Reason the data class is restricted or releasable.</x:v>
+      </x:c>
+      <x:c r="D128" s="51" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="129" ht="15" hidden="0" customHeight="1">
       <x:c r="A129" s="14" t="str">
-        <x:v>Raw_Data_Summary</x:v>
+        <x:v>Cohort_Metadata</x:v>
       </x:c>
       <x:c r="B129" s="15" t="str">
-        <x:v>included</x:v>
+        <x:v>variable</x:v>
       </x:c>
       <x:c r="C129" s="41" t="str">
-        <x:v>Whether records from the data class are included.</x:v>
+        <x:v>Aggregate design-metadata variable.</x:v>
       </x:c>
       <x:c r="D129" s="16" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="130" ht="15" hidden="0" customHeight="1">
-      <x:c r="A130" s="26" t="str">
-        <x:v>Raw_Data_Summary</x:v>
-      </x:c>
-      <x:c r="B130" s="27" t="str">
-        <x:v>access</x:v>
-      </x:c>
-      <x:c r="C130" s="40" t="str">
-        <x:v>Permitted access route.</x:v>
-      </x:c>
-      <x:c r="D130" s="28" t="str">
+      <x:c r="A130" s="49" t="str">
+        <x:v>Cohort_Metadata</x:v>
+      </x:c>
+      <x:c r="B130" s="50" t="str">
+        <x:v>value</x:v>
+      </x:c>
+      <x:c r="C130" s="59" t="str">
+        <x:v>Released aggregate or design value.</x:v>
+      </x:c>
+      <x:c r="D130" s="51" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="131" ht="15" hidden="0" customHeight="1">
       <x:c r="A131" s="14" t="str">
-        <x:v>Raw_Data_Summary</x:v>
+        <x:v>Cohort_Metadata</x:v>
       </x:c>
       <x:c r="B131" s="15" t="str">
-        <x:v>privacy_rationale</x:v>
+        <x:v>unit</x:v>
       </x:c>
       <x:c r="C131" s="41" t="str">
-        <x:v>Reason the data class is restricted or releasable.</x:v>
+        <x:v>Measurement unit.</x:v>
       </x:c>
       <x:c r="D131" s="16" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="15" hidden="0" customHeight="1">
-      <x:c r="A132" s="26" t="str">
+      <x:c r="A132" s="49" t="str">
         <x:v>Cohort_Metadata</x:v>
       </x:c>
-      <x:c r="B132" s="27" t="str">
-        <x:v>variable</x:v>
-      </x:c>
-      <x:c r="C132" s="40" t="str">
-        <x:v>Aggregate design-metadata variable.</x:v>
-      </x:c>
-      <x:c r="D132" s="28" t="str">
+      <x:c r="B132" s="50" t="str">
+        <x:v>level</x:v>
+      </x:c>
+      <x:c r="C132" s="59" t="str">
+        <x:v>Granularity of the data class or metadata.</x:v>
+      </x:c>
+      <x:c r="D132" s="51" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="15" hidden="0" customHeight="1">
-      <x:c r="A133" s="14" t="str">
+      <x:c r="A133" s="17" t="str">
         <x:v>Cohort_Metadata</x:v>
       </x:c>
-      <x:c r="B133" s="15" t="str">
-        <x:v>value</x:v>
-      </x:c>
-      <x:c r="C133" s="41" t="str">
-        <x:v>Released aggregate or design value.</x:v>
-      </x:c>
-      <x:c r="D133" s="16" t="str">
+      <x:c r="B133" s="18" t="str">
+        <x:v>note</x:v>
+      </x:c>
+      <x:c r="C133" s="61" t="str">
+        <x:v>Interpretive or privacy note.</x:v>
+      </x:c>
+      <x:c r="D133" s="19" t="str">
         <x:v>metadata/aggregate</x:v>
       </x:c>
     </x:row>
     <x:row r="134" ht="15" hidden="0" customHeight="1">
-      <x:c r="A134" s="26" t="str">
-        <x:v>Cohort_Metadata</x:v>
-      </x:c>
-      <x:c r="B134" s="27" t="str">
-        <x:v>unit</x:v>
-      </x:c>
-      <x:c r="C134" s="40" t="str">
-        <x:v>Measurement unit.</x:v>
-      </x:c>
-      <x:c r="D134" s="28" t="str">
-        <x:v>metadata/aggregate</x:v>
-      </x:c>
+      <x:c r="A134"/>
+      <x:c r="B134"/>
+      <x:c r="C134"/>
+      <x:c r="D134"/>
     </x:row>
     <x:row r="135" ht="15" hidden="0" customHeight="1">
-      <x:c r="A135" s="14" t="str">
-        <x:v>Cohort_Metadata</x:v>
-      </x:c>
-      <x:c r="B135" s="15" t="str">
-        <x:v>level</x:v>
-      </x:c>
-      <x:c r="C135" s="41" t="str">
-        <x:v>Granularity of the data class or metadata.</x:v>
-      </x:c>
-      <x:c r="D135" s="16" t="str">
-        <x:v>metadata/aggregate</x:v>
-      </x:c>
+      <x:c r="A135"/>
+      <x:c r="B135"/>
+      <x:c r="C135"/>
+      <x:c r="D135"/>
     </x:row>
     <x:row r="136" ht="15" hidden="0" customHeight="1">
-      <x:c r="A136" s="29" t="str">
-        <x:v>Cohort_Metadata</x:v>
-      </x:c>
-      <x:c r="B136" s="30" t="str">
-        <x:v>note</x:v>
-      </x:c>
-      <x:c r="C136" s="42" t="str">
-        <x:v>Interpretive or privacy note.</x:v>
-      </x:c>
-      <x:c r="D136" s="31" t="str">
-        <x:v>metadata/aggregate</x:v>
-      </x:c>
+      <x:c r="A136"/>
+      <x:c r="B136"/>
+      <x:c r="C136"/>
+      <x:c r="D136"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R053c8b58fa7d461c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree6a59212d234fbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3423,223 +3437,185 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="8" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="8" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="28" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="23" t="str">
-        <x:v>outcome</x:v>
-      </x:c>
-      <x:c r="B1" s="24" t="str">
-        <x:v>series</x:v>
-      </x:c>
-      <x:c r="C1" s="24" t="str">
-        <x:v>comparator</x:v>
-      </x:c>
-      <x:c r="D1" s="24" t="str">
-        <x:v>estimate</x:v>
-      </x:c>
-      <x:c r="E1" s="24" t="str">
+      <x:c r="A1" s="46" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="B1" s="47" t="str">
+        <x:v>mean_ap</x:v>
+      </x:c>
+      <x:c r="C1" s="47" t="str">
+        <x:v>delta_ap</x:v>
+      </x:c>
+      <x:c r="D1" s="47" t="str">
         <x:v>ci_low</x:v>
       </x:c>
-      <x:c r="F1" s="24" t="str">
+      <x:c r="E1" s="47" t="str">
         <x:v>ci_high</x:v>
       </x:c>
-      <x:c r="G1" s="24" t="str">
-        <x:v>reference</x:v>
-      </x:c>
-      <x:c r="H1" s="24" t="str">
-        <x:v>p_value</x:v>
-      </x:c>
-      <x:c r="I1" s="24" t="str">
-        <x:v>adjusted_p</x:v>
-      </x:c>
-      <x:c r="J1" s="24" t="str">
+      <x:c r="F1" s="47" t="str">
+        <x:v>exact_p</x:v>
+      </x:c>
+      <x:c r="G1" s="47" t="str">
+        <x:v>bh_p</x:v>
+      </x:c>
+      <x:c r="H1" s="47" t="str">
         <x:v>n</x:v>
       </x:c>
-      <x:c r="K1" s="24" t="str">
+      <x:c r="I1" s="47" t="str">
         <x:v>analysis_unit</x:v>
       </x:c>
-      <x:c r="L1" s="24" t="str">
-        <x:v>test</x:v>
-      </x:c>
-      <x:c r="M1" s="24" t="str">
+      <x:c r="J1" s="47" t="str">
         <x:v>note</x:v>
       </x:c>
+      <x:c r="K1"/>
+      <x:c r="L1"/>
+      <x:c r="M1"/>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="26" t="str">
-        <x:v>Paired AP difference</x:v>
-      </x:c>
-      <x:c r="B2" s="27" t="str">
+      <x:c r="A2" s="49" t="str">
         <x:v>HyNaPT</x:v>
       </x:c>
-      <x:c r="C2" s="27" t="str">
-        <x:v>Pairwise PLV</x:v>
-      </x:c>
-      <x:c r="D2" s="32" t="n">
-        <x:v>0.06703873826790492</x:v>
-      </x:c>
-      <x:c r="E2" s="32" t="n">
-        <x:v>0.004908471158471308</x:v>
-      </x:c>
-      <x:c r="F2" s="32" t="n">
-        <x:v>0.1318926278582527</x:v>
-      </x:c>
-      <x:c r="G2" s="32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H2" s="32" t="n">
-        <x:v>0.09765625</x:v>
-      </x:c>
-      <x:c r="I2" s="32" t="n">
-        <x:v>0.09765625</x:v>
-      </x:c>
-      <x:c r="J2" s="27" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="K2" s="27" t="str">
-        <x:v>paired cohort aggregate</x:v>
-      </x:c>
-      <x:c r="L2" s="27" t="str">
-        <x:v>Exact two-sided sign-flip test</x:v>
-      </x:c>
-      <x:c r="M2" s="35" t="str">
-        <x:v>Three primary controls form one BH family.</x:v>
-      </x:c>
+      <x:c r="B2" s="52" t="n">
+        <x:v>0.7340024574191241</x:v>
+      </x:c>
+      <x:c r="C2" s="52"/>
+      <x:c r="D2" s="52"/>
+      <x:c r="E2" s="52"/>
+      <x:c r="F2" s="52"/>
+      <x:c r="G2" s="52"/>
+      <x:c r="H2" s="50" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I2" s="50" t="str">
+        <x:v>cohort aggregate</x:v>
+      </x:c>
+      <x:c r="J2" s="55" t="str">
+        <x:v>Reference row in current Supplementary Table S1; participant rows withheld.</x:v>
+      </x:c>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="14" t="str">
-        <x:v>Paired AP difference</x:v>
-      </x:c>
-      <x:c r="B3" s="15" t="str">
-        <x:v>HyNaPT</x:v>
-      </x:c>
-      <x:c r="C3" s="15" t="str">
+        <x:v>Pairwise PLV</x:v>
+      </x:c>
+      <x:c r="B3" s="53" t="n">
+        <x:v>0.6669637191512192</x:v>
+      </x:c>
+      <x:c r="C3" s="53" t="n">
+        <x:v>0.06703873826790492</x:v>
+      </x:c>
+      <x:c r="D3" s="53" t="n">
+        <x:v>0.004908471158471308</x:v>
+      </x:c>
+      <x:c r="E3" s="53" t="n">
+        <x:v>0.1318926278582527</x:v>
+      </x:c>
+      <x:c r="F3" s="53" t="n">
+        <x:v>0.09765625</x:v>
+      </x:c>
+      <x:c r="G3" s="53" t="n">
+        <x:v>0.09765625</x:v>
+      </x:c>
+      <x:c r="H3" s="15" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I3" s="15" t="str">
+        <x:v>paired cohort aggregate</x:v>
+      </x:c>
+      <x:c r="J3" s="36" t="str">
+        <x:v>HyNaPT minus comparator; exact two-sided sign-flip test.</x:v>
+      </x:c>
+      <x:c r="K3"/>
+      <x:c r="L3"/>
+      <x:c r="M3"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="49" t="str">
         <x:v>Topology only</x:v>
       </x:c>
-      <x:c r="D3" s="33" t="n">
+      <x:c r="B4" s="52" t="n">
+        <x:v>0.6695345364512031</x:v>
+      </x:c>
+      <x:c r="C4" s="52" t="n">
         <x:v>0.064467920967921</x:v>
       </x:c>
-      <x:c r="E3" s="33" t="n">
+      <x:c r="D4" s="52" t="n">
         <x:v>0.014425423881674065</x:v>
       </x:c>
-      <x:c r="F3" s="33" t="n">
+      <x:c r="E4" s="52" t="n">
         <x:v>0.11754761904761918</x:v>
       </x:c>
-      <x:c r="G3" s="33" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H3" s="33" t="n">
+      <x:c r="F4" s="52" t="n">
         <x:v>0.03125</x:v>
       </x:c>
-      <x:c r="I3" s="33" t="n">
+      <x:c r="G4" s="52" t="n">
         <x:v>0.09375</x:v>
       </x:c>
-      <x:c r="J3" s="15" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="K3" s="15" t="str">
+      <x:c r="H4" s="50" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I4" s="50" t="str">
         <x:v>paired cohort aggregate</x:v>
       </x:c>
-      <x:c r="L3" s="15" t="str">
-        <x:v>Exact two-sided sign-flip test</x:v>
-      </x:c>
-      <x:c r="M3" s="36" t="str">
-        <x:v>Three primary controls form one BH family.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="26" t="str">
-        <x:v>Paired AP difference</x:v>
-      </x:c>
-      <x:c r="B4" s="27" t="str">
-        <x:v>HyNaPT</x:v>
-      </x:c>
-      <x:c r="C4" s="27" t="str">
-        <x:v>Attribute permutation</x:v>
-      </x:c>
-      <x:c r="D4" s="32" t="n">
-        <x:v>0.053869630369630404</x:v>
-      </x:c>
-      <x:c r="E4" s="32" t="n">
-        <x:v>0.007044707375957539</x:v>
-      </x:c>
-      <x:c r="F4" s="32" t="n">
-        <x:v>0.10564453185703189</x:v>
-      </x:c>
-      <x:c r="G4" s="32" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H4" s="32" t="n">
-        <x:v>0.06640625</x:v>
-      </x:c>
-      <x:c r="I4" s="32" t="n">
-        <x:v>0.09765625</x:v>
-      </x:c>
-      <x:c r="J4" s="27" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="K4" s="27" t="str">
-        <x:v>paired cohort aggregate</x:v>
-      </x:c>
-      <x:c r="L4" s="27" t="str">
-        <x:v>Exact two-sided sign-flip test</x:v>
-      </x:c>
-      <x:c r="M4" s="35" t="str">
-        <x:v>Three primary controls form one BH family.</x:v>
-      </x:c>
+      <x:c r="J4" s="55" t="str">
+        <x:v>HyNaPT minus comparator; exact two-sided sign-flip test.</x:v>
+      </x:c>
+      <x:c r="K4"/>
+      <x:c r="L4"/>
+      <x:c r="M4"/>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="17" t="str">
-        <x:v>Paired AP difference</x:v>
-      </x:c>
-      <x:c r="B5" s="18" t="str">
-        <x:v>HyNaPT</x:v>
-      </x:c>
-      <x:c r="C5" s="18" t="str">
-        <x:v>Bivariate Granger</x:v>
-      </x:c>
-      <x:c r="D5" s="38" t="n">
-        <x:v>0.0683328924162258</x:v>
-      </x:c>
-      <x:c r="E5" s="38" t="n">
-        <x:v>-0.0287123977873977</x:v>
-      </x:c>
-      <x:c r="F5" s="38" t="n">
-        <x:v>0.182609229196729</x:v>
-      </x:c>
-      <x:c r="G5" s="38" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H5" s="38" t="n">
-        <x:v>0.296875</x:v>
-      </x:c>
-      <x:c r="I5" s="38"/>
-      <x:c r="J5" s="18" t="n">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="K5" s="18" t="str">
+        <x:v>Attribute permutation</x:v>
+      </x:c>
+      <x:c r="B5" s="54" t="n">
+        <x:v>0.6801328270494937</x:v>
+      </x:c>
+      <x:c r="C5" s="54" t="n">
+        <x:v>0.053869630369630404</x:v>
+      </x:c>
+      <x:c r="D5" s="54" t="n">
+        <x:v>0.007044707375957539</x:v>
+      </x:c>
+      <x:c r="E5" s="54" t="n">
+        <x:v>0.10564453185703189</x:v>
+      </x:c>
+      <x:c r="F5" s="54" t="n">
+        <x:v>0.06640625</x:v>
+      </x:c>
+      <x:c r="G5" s="54" t="n">
+        <x:v>0.09765625</x:v>
+      </x:c>
+      <x:c r="H5" s="18" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I5" s="18" t="str">
         <x:v>paired cohort aggregate</x:v>
       </x:c>
-      <x:c r="L5" s="18" t="str">
-        <x:v>Exact two-sided sign-flip test</x:v>
-      </x:c>
-      <x:c r="M5" s="39" t="str">
-        <x:v>Granger was evaluated separately from the three-control BH family.</x:v>
-      </x:c>
+      <x:c r="J5" s="39" t="str">
+        <x:v>HyNaPT minus comparator; exact two-sided sign-flip test.</x:v>
+      </x:c>
+      <x:c r="K5"/>
+      <x:c r="L5"/>
+      <x:c r="M5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4380,7 +4356,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e11cb297ea446c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab24094c7cc645d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4724,7 +4700,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc699e1bcc15e469d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f258473603743ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5204,7 +5180,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R63156bdffdbb491e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cc63626949d4d66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5638,7 +5614,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ff4dff3e16b4b4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a7c6aa404194fd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7244,7 +7220,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03d7c1e184724193"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fbf123ec04a42fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8282,7 +8258,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e4bd84d50a04ed3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R291af43be28a42ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9366,7 +9342,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4f2f54fdb9d4755"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4db315aceaff4ee2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9555,7 +9531,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bfa18200989427d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d620e73fd3a4584"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>